<commit_message>
Actualizar README y mejoras del proyecto
</commit_message>
<xml_diff>
--- a/Template_llenado.xlsx
+++ b/Template_llenado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\programacion\Proyecto-Analitica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_BFF74F220C45C5CF2D0584A6F8021E8047ED04A0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4659C1-6591-4223-B80C-AF814AF7F553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,28 +73,28 @@
     <t>bases de datos donde escribe:</t>
   </si>
   <si>
+    <t>root</t>
+  </si>
+  <si>
+    <t>Escribe datos en Bases de datos</t>
+  </si>
+  <si>
+    <t>bases de datos consultadas:</t>
+  </si>
+  <si>
+    <t>Lee datos de bases de datos</t>
+  </si>
+  <si>
+    <t>Servidor donde está desplegada la solución</t>
+  </si>
+  <si>
+    <t>localhost / Windows 11</t>
+  </si>
+  <si>
+    <t>En desarrollo</t>
+  </si>
+  <si>
     <t>peliculas_db</t>
-  </si>
-  <si>
-    <t>root</t>
-  </si>
-  <si>
-    <t>Escribe datos en Bases de datos</t>
-  </si>
-  <si>
-    <t>bases de datos consultadas:</t>
-  </si>
-  <si>
-    <t>Lee datos de bases de datos</t>
-  </si>
-  <si>
-    <t>Servidor donde está desplegada la solución</t>
-  </si>
-  <si>
-    <t>localhost / Windows 11</t>
-  </si>
-  <si>
-    <t>En desarrollo</t>
   </si>
 </sst>
 </file>
@@ -434,6 +434,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -447,11 +452,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -783,13 +783,13 @@
       <c r="B3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="33"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="28"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
@@ -831,13 +831,13 @@
       <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="33" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="31" t="s">
         <v>12</v>
       </c>
       <c r="F7" s="12"/>
@@ -890,16 +890,16 @@
         <v>16</v>
       </c>
       <c r="E12" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="15" t="s">
         <v>17</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>18</v>
       </c>
       <c r="G12" s="4"/>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B13" s="20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -927,19 +927,19 @@
       <c r="B16" s="22"/>
       <c r="C16" s="23"/>
       <c r="D16" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E16" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="15" t="s">
         <v>17</v>
-      </c>
-      <c r="F16" s="15" t="s">
-        <v>18</v>
       </c>
       <c r="G16" s="4"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B17" s="20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
@@ -981,17 +981,17 @@
     </row>
     <row r="22" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="26" t="s">
+      <c r="D22" s="30"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="D22" s="27"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="G22" s="27"/>
+      <c r="G22" s="30"/>
     </row>
     <row r="23" spans="2:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="2"/>

</xml_diff>